<commit_message>
Guide and updated code
pushing the guide PDF and updated code, which cleaned up library dependencies and stored them in global.r
</commit_message>
<xml_diff>
--- a/supplemental/Analysis Output.xlsx
+++ b/supplemental/Analysis Output.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mdinw\Desktop\PPCORR Project\PPCORR Version Control\Old Versions\12-03-2023\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mdinw\Desktop\PPCORR Project\PPCORR Version Control\PCC\supplemental\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C39861D0-DE85-486F-A29B-339DA2361954}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6CC49CB3-9EFD-40B9-BC45-0D2E8652E624}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Figure 2B" sheetId="2" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="Figure 5CD" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -478,15 +479,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>55245</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>533093</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>114454</xdr:rowOff>
+      <xdr:colOff>133177</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>86592</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>4889</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>105795</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -509,8 +510,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="845820" y="4981575"/>
-          <a:ext cx="11450648" cy="1105054"/>
+          <a:off x="921154" y="5178137"/>
+          <a:ext cx="11388303" cy="1110249"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -700,16 +701,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>28575</xdr:colOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>574205</xdr:colOff>
       <xdr:row>32</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>58769</xdr:colOff>
+      <xdr:rowOff>66439</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>604398</xdr:colOff>
       <xdr:row>38</xdr:row>
-      <xdr:rowOff>97315</xdr:rowOff>
+      <xdr:rowOff>116129</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -732,8 +733,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="895350" y="5838825"/>
-          <a:ext cx="11599259" cy="1139350"/>
+          <a:off x="837612" y="5786143"/>
+          <a:ext cx="11648342" cy="1122134"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>